<commit_message>
EIKF.IC check D&A + Excel update
</commit_message>
<xml_diff>
--- a/data/isx_xlsx/EIKF.IC.xlsx
+++ b/data/isx_xlsx/EIKF.IC.xlsx
@@ -2910,9 +2910,15 @@
       <c r="H44" s="17"/>
       <c r="I44" s="17"/>
       <c r="J44" s="17"/>
-      <c r="K44" s="17"/>
-      <c r="L44" s="17"/>
-      <c r="M44" s="17"/>
+      <c r="K44" s="16">
+        <v>22.38</v>
+      </c>
+      <c r="L44" s="16">
+        <v>23.23</v>
+      </c>
+      <c r="M44" s="16">
+        <v>14.7</v>
+      </c>
       <c r="N44" s="16">
         <v>10.11</v>
       </c>

</xml_diff>